<commit_message>
Changes in some design
</commit_message>
<xml_diff>
--- a/BookCardReport.xlsx
+++ b/BookCardReport.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Svgu library\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{55FCDDF1-6563-44C3-988F-0434A699E8A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08112538-DB84-4D70-9070-ECBF0D18D0D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -133,19 +133,19 @@
     <t>2201BCA</t>
   </si>
   <si>
-    <t>title</t>
-  </si>
-  <si>
     <t>author</t>
   </si>
   <si>
     <t>class no</t>
   </si>
   <si>
-    <t>book no</t>
-  </si>
-  <si>
     <t>acc no</t>
+  </si>
+  <si>
+    <t>Title</t>
+  </si>
+  <si>
+    <t>Book No</t>
   </si>
 </sst>
 </file>
@@ -523,19 +523,19 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="C1" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>39</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>40</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>41</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="15.75" customHeight="1">
@@ -546,7 +546,7 @@
         <v>0</v>
       </c>
       <c r="D2" s="4">
-        <v>6.7</v>
+        <v>6.7854580000000002</v>
       </c>
       <c r="E2" t="s">
         <v>1</v>

</xml_diff>